<commit_message>
change questions for adult and add version in criteria
</commit_message>
<xml_diff>
--- a/data/adult.xlsx
+++ b/data/adult.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ecosenza/s/DifussionCompass/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stani\Documents\library\DiffusionCompass\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF54B4B-FD2B-BC41-865D-B13993F277A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0B47481-5520-4407-90D0-5DA4F6BEB32D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pipelines" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1157" uniqueCount="275">
   <si>
     <t>criterion_id</t>
   </si>
@@ -803,6 +803,54 @@
   </si>
   <si>
     <t>brainlife</t>
+  </si>
+  <si>
+    <t>DTI model</t>
+  </si>
+  <si>
+    <t>Inter-site harmonization support</t>
+  </si>
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>version use for this comparaison</t>
+  </si>
+  <si>
+    <t>1.2.11</t>
+  </si>
+  <si>
+    <t>0.4.0</t>
+  </si>
+  <si>
+    <t>6.0.0</t>
+  </si>
+  <si>
+    <t>23a</t>
+  </si>
+  <si>
+    <t>0.2.3</t>
+  </si>
+  <si>
+    <t>0.6.0</t>
+  </si>
+  <si>
+    <t>1.1.0</t>
+  </si>
+  <si>
+    <t>26.0.0</t>
+  </si>
+  <si>
+    <t>0.1.1</t>
+  </si>
+  <si>
+    <t>4.1.0</t>
+  </si>
+  <si>
+    <t>2.4.4</t>
+  </si>
+  <si>
+    <t>FreeSurfer 7.3</t>
   </si>
 </sst>
 </file>
@@ -1175,15 +1223,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O73"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:O74"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="15" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1230,7 +1278,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>14</v>
       </c>
@@ -1249,7 +1297,7 @@
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
     </row>
-    <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>15</v>
       </c>
@@ -1296,7 +1344,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>30</v>
       </c>
@@ -1315,7 +1363,7 @@
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
     </row>
-    <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>31</v>
       </c>
@@ -1362,7 +1410,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>34</v>
       </c>
@@ -1409,7 +1457,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>37</v>
       </c>
@@ -1456,7 +1504,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>39</v>
       </c>
@@ -1503,7 +1551,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>41</v>
       </c>
@@ -1522,7 +1570,7 @@
       <c r="N9" s="7"/>
       <c r="O9" s="7"/>
     </row>
-    <row r="10" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>42</v>
       </c>
@@ -1569,7 +1617,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>47</v>
       </c>
@@ -1616,7 +1664,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
@@ -1663,7 +1711,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>51</v>
       </c>
@@ -1710,7 +1758,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>55</v>
       </c>
@@ -1757,7 +1805,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>57</v>
       </c>
@@ -1804,7 +1852,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>59</v>
       </c>
@@ -1851,7 +1899,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>61</v>
       </c>
@@ -1898,7 +1946,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>63</v>
       </c>
@@ -1945,7 +1993,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>65</v>
       </c>
@@ -1992,7 +2040,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>71</v>
       </c>
@@ -2039,7 +2087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>73</v>
       </c>
@@ -2086,7 +2134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>75</v>
       </c>
@@ -2133,7 +2181,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>77</v>
       </c>
@@ -2180,836 +2228,836 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="7" t="s">
+    <row r="24" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="J24" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="K24" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="L24" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="M24" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="N24" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="O24" s="5" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
-      <c r="L24" s="7"/>
-      <c r="M24" s="7"/>
-      <c r="N24" s="7"/>
-      <c r="O24" s="7"/>
-    </row>
-    <row r="25" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="7"/>
+      <c r="N25" s="7"/>
+      <c r="O25" s="7"/>
+    </row>
+    <row r="26" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B26" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C25" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I25" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K25" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L25" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M25" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N25" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O25" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
+      <c r="C26" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K26" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L26" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M26" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N26" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O26" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B27" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I26" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J26" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K26" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L26" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M26" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N26" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O26" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="3" t="s">
+      <c r="C27" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J27" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K27" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L27" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M27" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N27" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O27" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B28" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="N27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O27" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="3" t="s">
+      <c r="C28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="N28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O28" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B29" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C28" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H28" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I28" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J28" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K28" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L28" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M28" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="N28" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O28" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="3" t="s">
+      <c r="C29" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K29" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L29" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M29" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="N29" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O29" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B30" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="C29" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I29" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K29" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L29" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M29" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N29" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O29" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="3" t="s">
+      <c r="C30" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K30" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L30" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M30" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N30" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O30" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B31" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C31" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D31" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="E30" s="5" t="s">
+      <c r="E31" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F30" s="5" t="s">
+      <c r="F31" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="G30" s="5" t="s">
+      <c r="G31" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="H30" s="5" t="s">
+      <c r="H31" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="I30" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J30" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K30" s="5" t="s">
+      <c r="I31" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J31" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K31" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="L30" s="5" t="s">
+      <c r="L31" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="M30" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N30" s="5" t="s">
+      <c r="M31" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N31" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="O30" s="5" t="s">
+      <c r="O31" s="5" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="31" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="3" t="s">
+    <row r="32" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B32" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C32" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="D31" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H31" s="5" t="s">
+      <c r="D32" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H32" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="I31" s="5" t="s">
+      <c r="I32" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="J31" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K31" s="5" t="s">
+      <c r="J32" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K32" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="L31" s="5" t="s">
+      <c r="L32" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="M31" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N31" s="5" t="s">
+      <c r="M32" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N32" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="O31" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="3" t="s">
+      <c r="O32" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B33" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C33" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="D33" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="E33" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="F32" s="5" t="s">
+      <c r="F33" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="G32" s="5" t="s">
+      <c r="G33" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="H32" s="5" t="s">
+      <c r="H33" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="I32" s="5" t="s">
+      <c r="I33" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="J32" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K32" s="5" t="s">
+      <c r="J33" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K33" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="L32" s="5" t="s">
+      <c r="L33" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="M32" s="5" t="s">
+      <c r="M33" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="N32" s="5" t="s">
+      <c r="N33" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="O32" s="5" t="s">
+      <c r="O33" s="5" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="33" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="3" t="s">
+    <row r="34" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B34" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H33" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I33" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J33" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K33" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L33" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M33" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="N33" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O33" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="3" t="s">
+      <c r="C34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="N34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O34" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B35" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D35" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="E34" s="5" t="s">
+      <c r="E35" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="F34" s="5" t="s">
+      <c r="F35" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="G34" s="5" t="s">
+      <c r="G35" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="H34" s="5" t="s">
+      <c r="H35" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="I34" s="5" t="s">
+      <c r="I35" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="J34" s="5" t="s">
+      <c r="J35" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="K34" s="5" t="s">
+      <c r="K35" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="L34" s="5" t="s">
+      <c r="L35" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="M34" s="5" t="s">
+      <c r="M35" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="N34" s="5" t="s">
+      <c r="N35" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="O34" s="5" t="s">
+      <c r="O35" s="5" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="35" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="3" t="s">
+    <row r="36" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B36" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="C35" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E35" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G35" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H35" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I35" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J35" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K35" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L35" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M35" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N35" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O35" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="3" t="s">
+      <c r="C36" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J36" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L36" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M36" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N36" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O36" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B37" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="C36" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D36" s="5" t="s">
+      <c r="C37" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D37" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="E36" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G36" s="5" t="s">
+      <c r="E37" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G37" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="H36" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I36" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J36" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K36" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="L36" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M36" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N36" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O36" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="3" t="s">
+      <c r="H37" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J37" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K37" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L37" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M37" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N37" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O37" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B38" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C37" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G37" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I37" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J37" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K37" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L37" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M37" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N37" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O37" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="3" t="s">
+      <c r="C38" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I38" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J38" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K38" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L38" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M38" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N38" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O38" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B39" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="C38" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G38" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H38" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I38" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J38" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K38" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L38" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M38" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N38" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O38" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="3" t="s">
+      <c r="C39" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I39" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J39" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K39" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L39" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M39" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N39" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O39" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B40" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C39" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G39" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H39" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I39" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J39" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K39" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L39" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M39" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="N39" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O39" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="3" t="s">
+      <c r="C40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="N40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O40" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B41" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="C40" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E40" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G40" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H40" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I40" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J40" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K40" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L40" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M40" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N40" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O40" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="3" t="s">
+      <c r="C41" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H41" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I41" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J41" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K41" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L41" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M41" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N41" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O41" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B42" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C42" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="D42" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="F41" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="G41" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="H41" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="I41" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="J41" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="K41" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="L41" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="M41" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="N41" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="O41" s="5" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>145</v>
       </c>
       <c r="E42" s="5" t="s">
         <v>96</v>
@@ -3021,1304 +3069,1351 @@
         <v>96</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="I42" s="5" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="J42" s="5" t="s">
         <v>96</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="L42" s="5" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="M42" s="5" t="s">
         <v>96</v>
       </c>
       <c r="N42" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="O42" s="5" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="H43" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="I43" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="J43" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="K43" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="L43" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="M43" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="N43" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="O42" s="5" t="s">
+      <c r="O43" s="5" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="43" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="7" t="s">
+    <row r="44" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="B43" s="7"/>
-      <c r="C43" s="7"/>
-      <c r="D43" s="7"/>
-      <c r="E43" s="7"/>
-      <c r="F43" s="7"/>
-      <c r="G43" s="7"/>
-      <c r="H43" s="7"/>
-      <c r="I43" s="7"/>
-      <c r="J43" s="7"/>
-      <c r="K43" s="7"/>
-      <c r="L43" s="7"/>
-      <c r="M43" s="7"/>
-      <c r="N43" s="7"/>
-      <c r="O43" s="7"/>
-    </row>
-    <row r="44" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="3" t="s">
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7"/>
+      <c r="F44" s="7"/>
+      <c r="G44" s="7"/>
+      <c r="H44" s="7"/>
+      <c r="I44" s="7"/>
+      <c r="J44" s="7"/>
+      <c r="K44" s="7"/>
+      <c r="L44" s="7"/>
+      <c r="M44" s="7"/>
+      <c r="N44" s="7"/>
+      <c r="O44" s="7"/>
+    </row>
+    <row r="45" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="B45" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="C44" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E44" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G44" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H44" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I44" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J44" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K44" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L44" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M44" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N44" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O44" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="3" t="s">
+      <c r="C45" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H45" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I45" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J45" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K45" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L45" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M45" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N45" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O45" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="B45" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D45" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E45" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G45" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H45" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I45" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J45" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K45" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L45" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M45" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="N45" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O45" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="3" t="s">
+      <c r="B46" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="N46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O46" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B47" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C46" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D46" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E46" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F46" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G46" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H46" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I46" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J46" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K46" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="L46" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M46" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N46" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O46" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="7" t="s">
+      <c r="C47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O47" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="B47" s="7"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="7"/>
-      <c r="F47" s="7"/>
-      <c r="G47" s="7"/>
-      <c r="H47" s="7"/>
-      <c r="I47" s="7"/>
-      <c r="J47" s="7"/>
-      <c r="K47" s="7"/>
-      <c r="L47" s="7"/>
-      <c r="M47" s="7"/>
-      <c r="N47" s="7"/>
-      <c r="O47" s="7"/>
-    </row>
-    <row r="48" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="3" t="s">
+      <c r="B48" s="7"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="7"/>
+      <c r="J48" s="7"/>
+      <c r="K48" s="7"/>
+      <c r="L48" s="7"/>
+      <c r="M48" s="7"/>
+      <c r="N48" s="7"/>
+      <c r="O48" s="7"/>
+    </row>
+    <row r="49" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="B48" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E48" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F48" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G48" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H48" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I48" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J48" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K48" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L48" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M48" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="N48" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O48" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="3" t="s">
+      <c r="B49" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F49" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G49" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H49" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I49" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J49" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K49" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L49" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M49" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="N49" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O49" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="B50" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="C49" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D49" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E49" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F49" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G49" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H49" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I49" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J49" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K49" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L49" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M49" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N49" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O49" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="3" t="s">
+      <c r="C50" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I50" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J50" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K50" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L50" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M50" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N50" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O50" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B51" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="C50" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D50" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E50" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F50" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G50" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H50" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I50" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J50" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K50" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L50" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M50" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N50" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O50" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="51" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="3" t="s">
+      <c r="C51" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F51" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H51" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I51" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J51" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K51" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L51" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M51" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N51" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O51" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B52" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="C51" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D51" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E51" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F51" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G51" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H51" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I51" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J51" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K51" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L51" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M51" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N51" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O51" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="3" t="s">
+      <c r="C52" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F52" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G52" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H52" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I52" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J52" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K52" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L52" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M52" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N52" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O52" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B53" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="C52" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E52" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F52" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G52" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H52" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I52" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J52" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K52" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L52" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M52" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N52" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O52" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="7" t="s">
+      <c r="C53" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F53" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G53" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H53" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I53" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J53" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K53" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L53" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M53" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N53" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O53" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="B53" s="7"/>
-      <c r="C53" s="7"/>
-      <c r="D53" s="7"/>
-      <c r="E53" s="7"/>
-      <c r="F53" s="7"/>
-      <c r="G53" s="7"/>
-      <c r="H53" s="7"/>
-      <c r="I53" s="7"/>
-      <c r="J53" s="7"/>
-      <c r="K53" s="7"/>
-      <c r="L53" s="7"/>
-      <c r="M53" s="7"/>
-      <c r="N53" s="7"/>
-      <c r="O53" s="7"/>
-    </row>
-    <row r="54" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="3" t="s">
+      <c r="B54" s="7"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
+      <c r="G54" s="7"/>
+      <c r="H54" s="7"/>
+      <c r="I54" s="7"/>
+      <c r="J54" s="7"/>
+      <c r="K54" s="7"/>
+      <c r="L54" s="7"/>
+      <c r="M54" s="7"/>
+      <c r="N54" s="7"/>
+      <c r="O54" s="7"/>
+    </row>
+    <row r="55" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="B55" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="C54" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E54" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F54" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G54" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H54" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I54" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J54" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K54" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L54" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M54" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N54" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O54" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="55" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="3" t="s">
+      <c r="C55" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G55" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H55" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I55" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J55" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K55" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L55" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M55" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N55" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O55" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B56" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="C55" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D55" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E55" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F55" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G55" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H55" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I55" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J55" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K55" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L55" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M55" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N55" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O55" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="56" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="3" t="s">
+      <c r="C56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M56" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O56" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B57" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="C56" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D56" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E56" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F56" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G56" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H56" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I56" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J56" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K56" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="L56" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M56" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N56" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O56" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="3" t="s">
+      <c r="C57" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F57" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G57" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H57" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I57" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J57" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K57" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L57" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M57" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N57" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O57" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="B58" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="C57" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D57" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E57" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F57" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G57" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H57" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I57" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J57" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K57" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L57" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M57" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="N57" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O57" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="7" t="s">
+      <c r="C58" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F58" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G58" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H58" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I58" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J58" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K58" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L58" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M58" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="N58" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O58" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="59" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="B58" s="7"/>
-      <c r="C58" s="7"/>
-      <c r="D58" s="7"/>
-      <c r="E58" s="7"/>
-      <c r="F58" s="7"/>
-      <c r="G58" s="7"/>
-      <c r="H58" s="7"/>
-      <c r="I58" s="7"/>
-      <c r="J58" s="7"/>
-      <c r="K58" s="7"/>
-      <c r="L58" s="7"/>
-      <c r="M58" s="7"/>
-      <c r="N58" s="7"/>
-      <c r="O58" s="7"/>
-    </row>
-    <row r="59" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="3" t="s">
+      <c r="B59" s="7"/>
+      <c r="C59" s="7"/>
+      <c r="D59" s="7"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="7"/>
+      <c r="G59" s="7"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="7"/>
+      <c r="J59" s="7"/>
+      <c r="K59" s="7"/>
+      <c r="L59" s="7"/>
+      <c r="M59" s="7"/>
+      <c r="N59" s="7"/>
+      <c r="O59" s="7"/>
+    </row>
+    <row r="60" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="B60" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C59" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D59" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E59" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F59" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G59" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H59" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I59" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J59" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K59" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L59" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M59" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N59" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O59" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="60" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="3" t="s">
+      <c r="C60" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G60" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H60" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I60" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J60" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K60" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L60" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M60" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N60" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O60" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="B61" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="C60" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D60" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E60" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F60" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G60" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H60" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I60" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J60" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K60" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L60" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M60" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N60" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O60" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="61" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="3" t="s">
+      <c r="C61" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F61" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G61" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H61" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I61" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J61" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K61" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L61" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M61" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N61" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O61" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B62" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C61" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D61" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E61" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F61" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G61" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H61" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I61" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J61" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K61" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="L61" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M61" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N61" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O61" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="62" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="7" t="s">
+      <c r="C62" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E62" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F62" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G62" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H62" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I62" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J62" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K62" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L62" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M62" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N62" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O62" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="63" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="B62" s="7"/>
-      <c r="C62" s="7"/>
-      <c r="D62" s="7"/>
-      <c r="E62" s="7"/>
-      <c r="F62" s="7"/>
-      <c r="G62" s="7"/>
-      <c r="H62" s="7"/>
-      <c r="I62" s="7"/>
-      <c r="J62" s="7"/>
-      <c r="K62" s="7"/>
-      <c r="L62" s="7"/>
-      <c r="M62" s="7"/>
-      <c r="N62" s="7"/>
-      <c r="O62" s="7"/>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A63" s="3" t="s">
+      <c r="B63" s="7"/>
+      <c r="C63" s="7"/>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7"/>
+      <c r="G63" s="7"/>
+      <c r="H63" s="7"/>
+      <c r="I63" s="7"/>
+      <c r="J63" s="7"/>
+      <c r="K63" s="7"/>
+      <c r="L63" s="7"/>
+      <c r="M63" s="7"/>
+      <c r="N63" s="7"/>
+      <c r="O63" s="7"/>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="B63" s="4" t="s">
+      <c r="B64" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="C63" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D63" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E63" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F63" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G63" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H63" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I63" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J63" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K63" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L63" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M63" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N63" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O63" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A64" s="3" t="s">
+      <c r="C64" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E64" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F64" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G64" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H64" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I64" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J64" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K64" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L64" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M64" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N64" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O64" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A65" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="B64" s="4" t="s">
+      <c r="B65" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="C64" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D64" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E64" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F64" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G64" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H64" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I64" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J64" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K64" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L64" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M64" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N64" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O64" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A65" s="3" t="s">
+      <c r="C65" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D65" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F65" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G65" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H65" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I65" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J65" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K65" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L65" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M65" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N65" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O65" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A66" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="B65" s="4" t="s">
+      <c r="B66" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C65" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D65" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E65" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F65" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G65" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H65" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I65" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J65" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K65" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L65" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M65" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N65" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O65" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="66" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="7" t="s">
+      <c r="C66" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F66" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G66" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H66" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I66" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J66" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K66" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L66" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M66" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N66" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O66" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="B66" s="7"/>
-      <c r="C66" s="7"/>
-      <c r="D66" s="7"/>
-      <c r="E66" s="7"/>
-      <c r="F66" s="7"/>
-      <c r="G66" s="7"/>
-      <c r="H66" s="7"/>
-      <c r="I66" s="7"/>
-      <c r="J66" s="7"/>
-      <c r="K66" s="7"/>
-      <c r="L66" s="7"/>
-      <c r="M66" s="7"/>
-      <c r="N66" s="7"/>
-      <c r="O66" s="7"/>
-    </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A67" s="3" t="s">
+      <c r="B67" s="7"/>
+      <c r="C67" s="7"/>
+      <c r="D67" s="7"/>
+      <c r="E67" s="7"/>
+      <c r="F67" s="7"/>
+      <c r="G67" s="7"/>
+      <c r="H67" s="7"/>
+      <c r="I67" s="7"/>
+      <c r="J67" s="7"/>
+      <c r="K67" s="7"/>
+      <c r="L67" s="7"/>
+      <c r="M67" s="7"/>
+      <c r="N67" s="7"/>
+      <c r="O67" s="7"/>
+    </row>
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A68" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B68" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="C67" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D67" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E67" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F67" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G67" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H67" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I67" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J67" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K67" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="L67" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M67" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N67" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O67" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A68" s="3" t="s">
+      <c r="C68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O68" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A69" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="B68" s="4" t="s">
+      <c r="B69" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="C68" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D68" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E68" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F68" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G68" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H68" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I68" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J68" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K68" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L68" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M68" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N68" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O68" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A69" s="3" t="s">
+      <c r="C69" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F69" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G69" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H69" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I69" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J69" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K69" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L69" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M69" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N69" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O69" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A70" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="B69" s="4" t="s">
+      <c r="B70" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="C69" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D69" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E69" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F69" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G69" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H69" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I69" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J69" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K69" s="5" t="s">
+      <c r="C70" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F70" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G70" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H70" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I70" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J70" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K70" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="L69" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M69" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N69" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O69" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A70" s="3" t="s">
+      <c r="L70" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M70" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N70" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O70" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A71" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="B70" s="4" t="s">
+      <c r="B71" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="C70" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D70" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E70" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F70" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G70" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H70" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I70" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J70" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K70" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="L70" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M70" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N70" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O70" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A71" s="3" t="s">
+      <c r="C71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O71" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A72" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="B71" s="4" t="s">
+      <c r="B72" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C71" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D71" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E71" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F71" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G71" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H71" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I71" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J71" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K71" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="L71" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M71" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N71" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O71" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="72" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="7" t="s">
+      <c r="C72" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F72" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G72" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H72" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I72" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J72" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K72" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L72" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M72" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N72" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O72" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="B72" s="7"/>
-      <c r="C72" s="7"/>
-      <c r="D72" s="7"/>
-      <c r="E72" s="7"/>
-      <c r="F72" s="7"/>
-      <c r="G72" s="7"/>
-      <c r="H72" s="7"/>
-      <c r="I72" s="7"/>
-      <c r="J72" s="7"/>
-      <c r="K72" s="7"/>
-      <c r="L72" s="7"/>
-      <c r="M72" s="7"/>
-      <c r="N72" s="7"/>
-      <c r="O72" s="7"/>
-    </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A73" s="3" t="s">
+      <c r="B73" s="7"/>
+      <c r="C73" s="7"/>
+      <c r="D73" s="7"/>
+      <c r="E73" s="7"/>
+      <c r="F73" s="7"/>
+      <c r="G73" s="7"/>
+      <c r="H73" s="7"/>
+      <c r="I73" s="7"/>
+      <c r="J73" s="7"/>
+      <c r="K73" s="7"/>
+      <c r="L73" s="7"/>
+      <c r="M73" s="7"/>
+      <c r="N73" s="7"/>
+      <c r="O73" s="7"/>
+    </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A74" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="B73" s="4" t="s">
+      <c r="B74" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="C73" s="5" t="s">
+      <c r="C74" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="D73" s="5" t="s">
+      <c r="D74" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="E73" s="5" t="s">
+      <c r="E74" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="F73" s="5" t="s">
+      <c r="F74" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="G73" s="5" t="s">
+      <c r="G74" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="H73" s="5" t="s">
+      <c r="H74" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="I73" s="5" t="s">
+      <c r="I74" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="J73" s="5" t="s">
+      <c r="J74" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="K73" s="5" t="s">
+      <c r="K74" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="L73" s="5" t="s">
+      <c r="L74" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="M73" s="5" t="s">
+      <c r="M74" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="N73" s="5" t="s">
+      <c r="N74" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="O73" s="5" t="s">
+      <c r="O74" s="5" t="s">
         <v>211</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A73:O73"/>
+    <mergeCell ref="A48:O48"/>
+    <mergeCell ref="A54:O54"/>
+    <mergeCell ref="A59:O59"/>
+    <mergeCell ref="A63:O63"/>
+    <mergeCell ref="A67:O67"/>
     <mergeCell ref="A2:O2"/>
     <mergeCell ref="A4:O4"/>
     <mergeCell ref="A9:O9"/>
-    <mergeCell ref="A24:O24"/>
-    <mergeCell ref="A43:O43"/>
-    <mergeCell ref="A72:O72"/>
-    <mergeCell ref="A47:O47"/>
-    <mergeCell ref="A53:O53"/>
-    <mergeCell ref="A58:O58"/>
-    <mergeCell ref="A62:O62"/>
-    <mergeCell ref="A66:O66"/>
+    <mergeCell ref="A25:O25"/>
+    <mergeCell ref="A44:O44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -4328,7 +4423,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>
@@ -4336,7 +4431,7 @@
     <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>218</v>
       </c>
@@ -4350,7 +4445,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>15</v>
       </c>
@@ -4364,7 +4459,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>42</v>
       </c>
@@ -4378,7 +4473,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>47</v>
       </c>
@@ -4392,7 +4487,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>49</v>
       </c>
@@ -4406,7 +4501,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>55</v>
       </c>
@@ -4420,7 +4515,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>59</v>
       </c>
@@ -4434,7 +4529,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>63</v>
       </c>
@@ -4448,7 +4543,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>65</v>
       </c>
@@ -4462,7 +4557,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>71</v>
       </c>
@@ -4476,7 +4571,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>73</v>
       </c>
@@ -4490,7 +4585,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>80</v>
       </c>
@@ -4504,7 +4599,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>82</v>
       </c>
@@ -4518,7 +4613,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>84</v>
       </c>
@@ -4532,7 +4627,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>86</v>
       </c>
@@ -4546,7 +4641,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>88</v>
       </c>
@@ -4560,7 +4655,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>115</v>
       </c>
@@ -4574,7 +4669,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>122</v>
       </c>
@@ -4588,7 +4683,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>130</v>
       </c>
@@ -4602,7 +4697,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>132</v>
       </c>
@@ -4616,7 +4711,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>134</v>
       </c>
@@ -4630,7 +4725,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>158</v>
       </c>
@@ -4644,7 +4739,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>160</v>
       </c>
@@ -4658,7 +4753,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>162</v>
       </c>
@@ -4672,7 +4767,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>164</v>
       </c>
@@ -4686,7 +4781,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>167</v>
       </c>
@@ -4700,7 +4795,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>169</v>
       </c>
@@ -4714,7 +4809,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>171</v>
       </c>
@@ -4728,7 +4823,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>176</v>
       </c>
@@ -4742,7 +4837,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>178</v>
       </c>
@@ -4756,7 +4851,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>180</v>
       </c>
@@ -4770,7 +4865,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>34</v>
       </c>
@@ -4784,7 +4879,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>37</v>
       </c>
@@ -4798,7 +4893,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>39</v>
       </c>
@@ -4812,7 +4907,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>149</v>
       </c>
@@ -4826,7 +4921,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>153</v>
       </c>
@@ -4840,7 +4935,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>203</v>
       </c>
@@ -4854,7 +4949,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>31</v>
       </c>
@@ -4868,7 +4963,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>51</v>
       </c>
@@ -4882,7 +4977,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>57</v>
       </c>
@@ -4896,7 +4991,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>61</v>
       </c>
@@ -4910,7 +5005,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>90</v>
       </c>
@@ -4924,7 +5019,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>98</v>
       </c>
@@ -4938,7 +5033,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>104</v>
       </c>
@@ -4952,7 +5047,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>117</v>
       </c>
@@ -4966,7 +5061,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>128</v>
       </c>
@@ -4980,7 +5075,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>136</v>
       </c>
@@ -4994,7 +5089,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>140</v>
       </c>
@@ -5008,7 +5103,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>151</v>
       </c>
@@ -5022,7 +5117,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>156</v>
       </c>
@@ -5036,7 +5131,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>173</v>
       </c>
@@ -5050,7 +5145,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>183</v>
       </c>
@@ -5064,7 +5159,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>185</v>
       </c>
@@ -5078,7 +5173,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>187</v>
       </c>
@@ -5092,7 +5187,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>189</v>
       </c>
@@ -5106,7 +5201,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>192</v>
       </c>
@@ -5120,7 +5215,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>194</v>
       </c>
@@ -5134,7 +5229,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="58" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>196</v>
       </c>
@@ -5148,7 +5243,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>198</v>
       </c>
@@ -5162,7 +5257,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>200</v>
       </c>
@@ -5176,7 +5271,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>124</v>
       </c>
@@ -5190,7 +5285,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="62" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>75</v>
       </c>
@@ -5204,7 +5299,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>77</v>
       </c>
@@ -5218,7 +5313,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:4" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="8" t="s">
         <v>239</v>
       </c>

</xml_diff>